<commit_message>
Fantravel opti, IT, FR, ES, DE added
</commit_message>
<xml_diff>
--- a/club_names.xlsx
+++ b/club_names.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcuskarberg/Desktop/Football-Travel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3626CA73-17A3-B349-AB7E-E51BFB00DDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8821DC2A-C2CB-B647-884D-1E5C24BBCC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15720" xr2:uid="{11594A43-A07C-9749-950F-F6643440C8D3}"/>
+    <workbookView xWindow="34600" yWindow="-420" windowWidth="27040" windowHeight="15720" xr2:uid="{11594A43-A07C-9749-950F-F6643440C8D3}"/>
   </bookViews>
   <sheets>
     <sheet name="EN" sheetId="1" r:id="rId1"/>
@@ -38,41 +38,26 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
   <si>
     <t>Arsenal</t>
   </si>
   <si>
-    <t>Aston Villa</t>
-  </si>
-  <si>
     <t>Brentford</t>
   </si>
   <si>
     <t>Crystal Palace</t>
   </si>
   <si>
-    <t>Leeds United</t>
-  </si>
-  <si>
     <t>Manchester City</t>
   </si>
   <si>
     <t>Manchester United</t>
   </si>
   <si>
-    <t>Newcastle United</t>
-  </si>
-  <si>
-    <t>Nottingham Forest</t>
-  </si>
-  <si>
     <t>Tottenham</t>
   </si>
   <si>
-    <t>West Ham United</t>
-  </si>
-  <si>
     <t>Lille</t>
   </si>
   <si>
@@ -145,9 +130,6 @@
     <t>Barcelona</t>
   </si>
   <si>
-    <t>Burnley</t>
-  </si>
-  <si>
     <t>Chelsea</t>
   </si>
   <si>
@@ -164,6 +146,30 @@
   </si>
   <si>
     <t>Atletico Madrid</t>
+  </si>
+  <si>
+    <t>Dortmund</t>
+  </si>
+  <si>
+    <t>Bayern München</t>
+  </si>
+  <si>
+    <t>AC Milan</t>
+  </si>
+  <si>
+    <t>Inter</t>
+  </si>
+  <si>
+    <t>Atalanta</t>
+  </si>
+  <si>
+    <t>Lazio</t>
+  </si>
+  <si>
+    <t>Juventus</t>
+  </si>
+  <si>
+    <t>West Ham</t>
   </si>
 </sst>
 </file>
@@ -543,7 +549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E59EE5-AAB7-EA4D-80FE-08D6137F1C18}">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -565,32 +571,32 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -600,52 +606,72 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -665,98 +691,98 @@
   <sheetData>
     <row r="1" spans="1:2" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -776,33 +802,33 @@
   <sheetData>
     <row r="1" spans="1:2" ht="22" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>